<commit_message>
Fix workflow setup cache and remove unused pandas dependency
</commit_message>
<xml_diff>
--- a/tests/reports/test_report.xlsx
+++ b/tests/reports/test_report.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:09</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="K2" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:04</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="K3" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:04</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="K4" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:04</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="K5" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:04</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="K6" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:04</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="K7" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="K8" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="K9" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="K10" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="K11" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -1973,7 +1973,7 @@
       </c>
       <c r="K12" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="K13" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="K14" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="K15" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="K17" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="K18" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="K19" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="K20" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="K21" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2557,7 +2557,7 @@
       </c>
       <c r="K22" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="K23" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="K24" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="K25" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="K26" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="K27" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="K28" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="K29" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="K30" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="K31" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="K32" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="K33" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3254,7 +3254,7 @@
       </c>
       <c r="K34" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="K35" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3370,7 @@
       </c>
       <c r="K36" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3428,7 +3428,7 @@
       </c>
       <c r="K37" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3487,7 +3487,7 @@
       </c>
       <c r="K38" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="K39" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3604,7 +3604,7 @@
       </c>
       <c r="K40" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="K41" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="K42" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="K43" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="K44" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3898,7 +3898,7 @@
       </c>
       <c r="K45" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="K46" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:20</t>
         </is>
       </c>
     </row>
@@ -4015,7 +4015,7 @@
       </c>
       <c r="K47" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4073,7 @@
       </c>
       <c r="K48" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="K49" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="K50" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="K51" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="K52" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4367,7 +4367,7 @@
       </c>
       <c r="K53" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="K54" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:05</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4485,7 @@
       </c>
       <c r="K55" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4544,7 @@
       </c>
       <c r="K56" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4603,7 @@
       </c>
       <c r="K57" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="K58" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="K59" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="K60" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="K61" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4897,7 +4897,7 @@
       </c>
       <c r="K62" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="K63" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5014,7 +5014,7 @@
       </c>
       <c r="K64" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="K65" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="K66" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5188,7 @@
       </c>
       <c r="K67" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="K68" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5304,7 +5304,7 @@
       </c>
       <c r="K69" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="K70" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5422,7 +5422,7 @@
       </c>
       <c r="K71" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5481,7 +5481,7 @@
       </c>
       <c r="K72" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5540,7 +5540,7 @@
       </c>
       <c r="K73" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="K74" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5657,7 +5657,7 @@
       </c>
       <c r="K75" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5715,7 @@
       </c>
       <c r="K76" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="K77" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5833,7 +5833,7 @@
       </c>
       <c r="K78" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5892,7 +5892,7 @@
       </c>
       <c r="K79" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -5950,7 +5950,7 @@
       </c>
       <c r="K80" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6008,7 +6008,7 @@
       </c>
       <c r="K81" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6066,7 +6066,7 @@
       </c>
       <c r="K82" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="K83" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="K84" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6242,7 +6242,7 @@
       </c>
       <c r="K85" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="K86" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6360,7 +6360,7 @@
       </c>
       <c r="K87" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6419,7 +6419,7 @@
       </c>
       <c r="K88" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6478,7 +6478,7 @@
       </c>
       <c r="K89" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="K90" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="K91" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6655,7 +6655,7 @@
       </c>
       <c r="K92" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6714,7 +6714,7 @@
       </c>
       <c r="K93" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="K94" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:21</t>
         </is>
       </c>
     </row>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="K95" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -6888,7 +6888,7 @@
       </c>
       <c r="K96" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -6947,7 +6947,7 @@
       </c>
       <c r="K97" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7005,7 +7005,7 @@
       </c>
       <c r="K98" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="K99" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="K100" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:06</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="K101" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7239,7 +7239,7 @@
       </c>
       <c r="K102" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7297,7 @@
       </c>
       <c r="K103" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="K104" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7413,7 +7413,7 @@
       </c>
       <c r="K105" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7471,7 +7471,7 @@
       </c>
       <c r="K106" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7529,7 @@
       </c>
       <c r="K107" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7587,7 +7587,7 @@
       </c>
       <c r="K108" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7645,7 +7645,7 @@
       </c>
       <c r="K109" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="K110" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7762,7 @@
       </c>
       <c r="K111" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7820,7 +7820,7 @@
       </c>
       <c r="K112" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="K113" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7940,7 +7940,7 @@
       </c>
       <c r="K114" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -7998,7 +7998,7 @@
       </c>
       <c r="K115" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8057,7 +8057,7 @@
       </c>
       <c r="K116" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8116,7 +8116,7 @@
       </c>
       <c r="K117" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8175,7 +8175,7 @@
       </c>
       <c r="K118" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8233,7 +8233,7 @@
       </c>
       <c r="K119" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="K120" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8349,7 +8349,7 @@
       </c>
       <c r="K121" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8408,7 +8408,7 @@
       </c>
       <c r="K122" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8466,7 +8466,7 @@
       </c>
       <c r="K123" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="K124" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="K125" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8641,7 +8641,7 @@
       </c>
       <c r="K126" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8699,7 +8699,7 @@
       </c>
       <c r="K127" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8757,7 +8757,7 @@
       </c>
       <c r="K128" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8815,7 +8815,7 @@
       </c>
       <c r="K129" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8874,7 +8874,7 @@
       </c>
       <c r="K130" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="K131" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -8991,7 +8991,7 @@
       </c>
       <c r="K132" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="K133" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9107,7 +9107,7 @@
       </c>
       <c r="K134" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="K135" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9223,7 +9223,7 @@
       </c>
       <c r="K136" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9281,7 +9281,7 @@
       </c>
       <c r="K137" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9339,7 +9339,7 @@
       </c>
       <c r="K138" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9397,7 +9397,7 @@
       </c>
       <c r="K139" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9455,7 +9455,7 @@
       </c>
       <c r="K140" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9514,7 +9514,7 @@
       </c>
       <c r="K141" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9574,7 +9574,7 @@
       </c>
       <c r="K142" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9632,7 +9632,7 @@
       </c>
       <c r="K143" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:22</t>
         </is>
       </c>
     </row>
@@ -9690,7 +9690,7 @@
       </c>
       <c r="K144" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -9749,7 +9749,7 @@
       </c>
       <c r="K145" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -9808,7 +9808,7 @@
       </c>
       <c r="K146" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -9866,7 +9866,7 @@
       </c>
       <c r="K147" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -9924,7 +9924,7 @@
       </c>
       <c r="K148" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -9982,7 +9982,7 @@
       </c>
       <c r="K149" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:07</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10041,7 +10041,7 @@
       </c>
       <c r="K150" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10099,7 +10099,7 @@
       </c>
       <c r="K151" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10157,7 +10157,7 @@
       </c>
       <c r="K152" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10215,7 +10215,7 @@
       </c>
       <c r="K153" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10273,7 +10273,7 @@
       </c>
       <c r="K154" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10331,7 +10331,7 @@
       </c>
       <c r="K155" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10389,7 +10389,7 @@
       </c>
       <c r="K156" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10447,7 +10447,7 @@
       </c>
       <c r="K157" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10505,7 +10505,7 @@
       </c>
       <c r="K158" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10563,7 +10563,7 @@
       </c>
       <c r="K159" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10621,7 +10621,7 @@
       </c>
       <c r="K160" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10680,7 +10680,7 @@
       </c>
       <c r="K161" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10738,7 +10738,7 @@
       </c>
       <c r="K162" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="K163" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10855,7 +10855,7 @@
       </c>
       <c r="K164" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10913,7 +10913,7 @@
       </c>
       <c r="K165" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -10971,7 +10971,7 @@
       </c>
       <c r="K166" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11029,7 +11029,7 @@
       </c>
       <c r="K167" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="K168" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="K169" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11206,7 +11206,7 @@
       </c>
       <c r="K170" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11265,7 +11265,7 @@
       </c>
       <c r="K171" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11324,7 +11324,7 @@
       </c>
       <c r="K172" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11382,7 +11382,7 @@
       </c>
       <c r="K173" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11440,7 +11440,7 @@
       </c>
       <c r="K174" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="K175" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="K176" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="K177" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11674,7 +11674,7 @@
       </c>
       <c r="K178" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11732,7 +11732,7 @@
       </c>
       <c r="K179" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11790,7 +11790,7 @@
       </c>
       <c r="K180" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11849,7 +11849,7 @@
       </c>
       <c r="K181" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11907,7 +11907,7 @@
       </c>
       <c r="K182" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -11965,7 +11965,7 @@
       </c>
       <c r="K183" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -12023,7 +12023,7 @@
       </c>
       <c r="K184" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -12081,7 +12081,7 @@
       </c>
       <c r="K185" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -12139,7 +12139,7 @@
       </c>
       <c r="K186" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -12198,7 +12198,7 @@
       </c>
       <c r="K187" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -12257,7 +12257,7 @@
       </c>
       <c r="K188" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -12315,7 +12315,7 @@
       </c>
       <c r="K189" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -12374,7 +12374,7 @@
       </c>
       <c r="K190" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -12432,7 +12432,7 @@
       </c>
       <c r="K191" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:23</t>
         </is>
       </c>
     </row>
@@ -12490,7 +12490,7 @@
       </c>
       <c r="K192" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="K193" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>
@@ -12607,7 +12607,7 @@
       </c>
       <c r="K194" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>
@@ -12665,7 +12665,7 @@
       </c>
       <c r="K195" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>
@@ -12723,7 +12723,7 @@
       </c>
       <c r="K196" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>
@@ -12782,7 +12782,7 @@
       </c>
       <c r="K197" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>
@@ -12840,7 +12840,7 @@
       </c>
       <c r="K198" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:08</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>
@@ -12899,7 +12899,7 @@
       </c>
       <c r="K199" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:09</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>
@@ -12958,7 +12958,7 @@
       </c>
       <c r="K200" s="19" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:09</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>
@@ -13017,7 +13017,7 @@
       </c>
       <c r="K201" s="22" t="inlineStr">
         <is>
-          <t>2026-06-18 09:51:09</t>
+          <t>2026-06-18 10:39:24</t>
         </is>
       </c>
     </row>

</xml_diff>